<commit_message>
chore: order fill-price hardening, refreshed instruments and session data
- PROD10FEB / ENHANCED: get_order_executed_price() now takes the expected fill qty
  (or learns it from order-status filled_quantity) and keeps retrying while the
  trades endpoint returns a list that is empty or short of that qty — a non-empty
  trade_list is not proof of completeness on large multi-trade fills. Cancel is
  accepted on CANCELLATION_REQUESTED as well as CANCELLED. Spec 01 updated to match.
- Refreshed instrument.csv, OI snapshot/dashboard, VIX and trendline caches, Lakshmi
  trade log, and today's trade history; new .premium_pulse_verdicts.json cache.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lakshmi.xlsx
+++ b/Lakshmi.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1624"/>
+  <dimension ref="A1:I1717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="24.33203125" customWidth="1" style="1" min="1" max="1"/>
@@ -47231,6 +47231,3183 @@
       <c r="I1624" t="inlineStr">
         <is>
           <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:30:10</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1625" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="D1625" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="E1625" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1625" t="n">
+        <v>1657.5</v>
+      </c>
+      <c r="G1625" t="n">
+        <v>98676.5</v>
+      </c>
+      <c r="H1625" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1625" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:30:56</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1626" t="n">
+        <v>90.15000000000001</v>
+      </c>
+      <c r="D1626" t="n">
+        <v>91.65000000000001</v>
+      </c>
+      <c r="E1626" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1626" t="n">
+        <v>1657.5</v>
+      </c>
+      <c r="G1626" t="n">
+        <v>99615.75</v>
+      </c>
+      <c r="H1626" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1626" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:33:00</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>NIFTY2680424600PE</t>
+        </is>
+      </c>
+      <c r="C1627" t="n">
+        <v>140.13</v>
+      </c>
+      <c r="D1627" t="n">
+        <v>141.65</v>
+      </c>
+      <c r="E1627" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1627" t="n">
+        <v>1679.6</v>
+      </c>
+      <c r="G1627" t="n">
+        <v>154843.65</v>
+      </c>
+      <c r="H1627" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1627" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:49:35</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1628" t="n">
+        <v>128.23</v>
+      </c>
+      <c r="D1628" t="n">
+        <v>121.58</v>
+      </c>
+      <c r="E1628" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1628" t="n">
+        <v>-7348.25</v>
+      </c>
+      <c r="G1628" t="n">
+        <v>141694.15</v>
+      </c>
+      <c r="H1628" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1628" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:53:04</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1629" t="n">
+        <v>126.61</v>
+      </c>
+      <c r="D1629" t="n">
+        <v>120.15</v>
+      </c>
+      <c r="E1629" t="n">
+        <v>975</v>
+      </c>
+      <c r="F1629" t="n">
+        <v>-6298.5</v>
+      </c>
+      <c r="G1629" t="n">
+        <v>123444.75</v>
+      </c>
+      <c r="H1629" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1629" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:53:45</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1630" t="n">
+        <v>100</v>
+      </c>
+      <c r="D1630" t="n">
+        <v>102</v>
+      </c>
+      <c r="E1630" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1630" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G1630" t="n">
+        <v>110500</v>
+      </c>
+      <c r="H1630" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1630" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:53:58</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1631" t="n">
+        <v>103.39</v>
+      </c>
+      <c r="D1631" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="E1631" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1631" t="n">
+        <v>2221.05</v>
+      </c>
+      <c r="G1631" t="n">
+        <v>114245.95</v>
+      </c>
+      <c r="H1631" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1631" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:54:23</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1632" t="n">
+        <v>109.02</v>
+      </c>
+      <c r="D1632" t="n">
+        <v>111</v>
+      </c>
+      <c r="E1632" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1632" t="n">
+        <v>2187.9</v>
+      </c>
+      <c r="G1632" t="n">
+        <v>120467.1</v>
+      </c>
+      <c r="H1632" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1632" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:55:18</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1633" t="n">
+        <v>109.17</v>
+      </c>
+      <c r="D1633" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="E1633" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1633" t="n">
+        <v>-6762.6</v>
+      </c>
+      <c r="G1633" t="n">
+        <v>120632.85</v>
+      </c>
+      <c r="H1633" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1633" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:56:22</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1634" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="D1634" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="E1634" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1634" t="n">
+        <v>2762.5</v>
+      </c>
+      <c r="G1634" t="n">
+        <v>114478</v>
+      </c>
+      <c r="H1634" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1634" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:57:05</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1635" t="n">
+        <v>107.65</v>
+      </c>
+      <c r="D1635" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="E1635" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1635" t="n">
+        <v>2762.5</v>
+      </c>
+      <c r="G1635" t="n">
+        <v>118953.25</v>
+      </c>
+      <c r="H1635" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1635" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:57:49</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1636" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="D1636" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="E1636" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1636" t="n">
+        <v>2762.5</v>
+      </c>
+      <c r="G1636" t="n">
+        <v>121329</v>
+      </c>
+      <c r="H1636" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1636" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:57:56</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1637" t="n">
+        <v>117.29</v>
+      </c>
+      <c r="D1637" t="n">
+        <v>119.8</v>
+      </c>
+      <c r="E1637" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1637" t="n">
+        <v>2773.55</v>
+      </c>
+      <c r="G1637" t="n">
+        <v>129605.45</v>
+      </c>
+      <c r="H1637" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1637" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>2026-08-04 13:58:22</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1638" t="n">
+        <v>120.04</v>
+      </c>
+      <c r="D1638" t="n">
+        <v>114.69</v>
+      </c>
+      <c r="E1638" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1638" t="n">
+        <v>-5911.75</v>
+      </c>
+      <c r="G1638" t="n">
+        <v>132644.2</v>
+      </c>
+      <c r="H1638" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1638" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:00:14</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1639" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="D1639" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="E1639" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1639" t="n">
+        <v>2784.6</v>
+      </c>
+      <c r="G1639" t="n">
+        <v>119317.9</v>
+      </c>
+      <c r="H1639" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1639" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:01:05</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1640" t="n">
+        <v>109.06</v>
+      </c>
+      <c r="D1640" t="n">
+        <v>111.55</v>
+      </c>
+      <c r="E1640" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1640" t="n">
+        <v>2751.45</v>
+      </c>
+      <c r="G1640" t="n">
+        <v>120511.3</v>
+      </c>
+      <c r="H1640" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1640" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:03:45</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr">
+        <is>
+          <t>NIFTY2680424550PE</t>
+        </is>
+      </c>
+      <c r="C1641" t="n">
+        <v>111.33</v>
+      </c>
+      <c r="D1641" t="n">
+        <v>113.85</v>
+      </c>
+      <c r="E1641" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1641" t="n">
+        <v>2784.6</v>
+      </c>
+      <c r="G1641" t="n">
+        <v>123019.65</v>
+      </c>
+      <c r="H1641" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1641" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:44:52</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr">
+        <is>
+          <t>NIFTY2680424600PE</t>
+        </is>
+      </c>
+      <c r="C1642" t="n">
+        <v>143.63</v>
+      </c>
+      <c r="D1642" t="n">
+        <v>136.66</v>
+      </c>
+      <c r="E1642" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1642" t="n">
+        <v>-7701.85</v>
+      </c>
+      <c r="G1642" t="n">
+        <v>158711.15</v>
+      </c>
+      <c r="H1642" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1642" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:49:48</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1643" t="n">
+        <v>133.37</v>
+      </c>
+      <c r="D1643" t="n">
+        <v>136.35</v>
+      </c>
+      <c r="E1643" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1643" t="n">
+        <v>3292.9</v>
+      </c>
+      <c r="G1643" t="n">
+        <v>147373.85</v>
+      </c>
+      <c r="H1643" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1643" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:50:07</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1644" t="n">
+        <v>135.87</v>
+      </c>
+      <c r="D1644" t="n">
+        <v>137.35</v>
+      </c>
+      <c r="E1644" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1644" t="n">
+        <v>1635.4</v>
+      </c>
+      <c r="G1644" t="n">
+        <v>150136.35</v>
+      </c>
+      <c r="H1644" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1644" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:51:52</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1645" t="n">
+        <v>137.14</v>
+      </c>
+      <c r="D1645" t="n">
+        <v>132.67</v>
+      </c>
+      <c r="E1645" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1645" t="n">
+        <v>-4939.35</v>
+      </c>
+      <c r="G1645" t="n">
+        <v>151539.7</v>
+      </c>
+      <c r="H1645" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1645" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:52:55</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1646" t="n">
+        <v>135.92</v>
+      </c>
+      <c r="D1646" t="n">
+        <v>137.4</v>
+      </c>
+      <c r="E1646" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1646" t="n">
+        <v>1635.4</v>
+      </c>
+      <c r="G1646" t="n">
+        <v>150191.6</v>
+      </c>
+      <c r="H1646" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1646" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:54:03</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1647" t="n">
+        <v>137.28</v>
+      </c>
+      <c r="D1647" t="n">
+        <v>138.8</v>
+      </c>
+      <c r="E1647" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1647" t="n">
+        <v>1679.6</v>
+      </c>
+      <c r="G1647" t="n">
+        <v>151694.4</v>
+      </c>
+      <c r="H1647" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1647" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:54:29</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1648" t="n">
+        <v>139.1</v>
+      </c>
+      <c r="D1648" t="n">
+        <v>139.21</v>
+      </c>
+      <c r="E1648" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1648" t="n">
+        <v>121.55</v>
+      </c>
+      <c r="G1648" t="n">
+        <v>153705.5</v>
+      </c>
+      <c r="H1648" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1648" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:55:14</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1649" t="n">
+        <v>140.4</v>
+      </c>
+      <c r="D1649" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="E1649" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1649" t="n">
+        <v>2762.5</v>
+      </c>
+      <c r="G1649" t="n">
+        <v>155142</v>
+      </c>
+      <c r="H1649" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1649" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>2026-08-04 14:55:45</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr">
+        <is>
+          <t>NIFTY2680424350CE</t>
+        </is>
+      </c>
+      <c r="C1650" t="n">
+        <v>140.68</v>
+      </c>
+      <c r="D1650" t="n">
+        <v>143.2</v>
+      </c>
+      <c r="E1650" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F1650" t="n">
+        <v>2784.6</v>
+      </c>
+      <c r="G1650" t="n">
+        <v>155451.4</v>
+      </c>
+      <c r="H1650" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1650" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>2026-08-06 09:44:09</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr">
+        <is>
+          <t>SENSEX2680678800CE</t>
+        </is>
+      </c>
+      <c r="C1651" t="n">
+        <v>297.85</v>
+      </c>
+      <c r="D1651" t="n">
+        <v>301.85</v>
+      </c>
+      <c r="E1651" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1651" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G1651" t="n">
+        <v>297850</v>
+      </c>
+      <c r="H1651" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1651" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>2026-08-06 09:44:51</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>SENSEX2680678800CE</t>
+        </is>
+      </c>
+      <c r="C1652" t="n">
+        <v>300.94</v>
+      </c>
+      <c r="D1652" t="n">
+        <v>304.95</v>
+      </c>
+      <c r="E1652" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1652" t="n">
+        <v>4010</v>
+      </c>
+      <c r="G1652" t="n">
+        <v>300940</v>
+      </c>
+      <c r="H1652" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1652" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:02:38</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1653" t="n">
+        <v>224.43</v>
+      </c>
+      <c r="D1653" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="E1653" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1653" t="n">
+        <v>4070</v>
+      </c>
+      <c r="G1653" t="n">
+        <v>224430</v>
+      </c>
+      <c r="H1653" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1653" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:02:59</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1654" t="n">
+        <v>233.2</v>
+      </c>
+      <c r="D1654" t="n">
+        <v>238.57</v>
+      </c>
+      <c r="E1654" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1654" t="n">
+        <v>5370</v>
+      </c>
+      <c r="G1654" t="n">
+        <v>233200</v>
+      </c>
+      <c r="H1654" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1654" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:50:51</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1655" t="n">
+        <v>236.53</v>
+      </c>
+      <c r="D1655" t="n">
+        <v>239.55</v>
+      </c>
+      <c r="E1655" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1655" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G1655" t="n">
+        <v>236530</v>
+      </c>
+      <c r="H1655" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1655" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:51:38</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1656" t="n">
+        <v>243.76</v>
+      </c>
+      <c r="D1656" t="n">
+        <v>246.75</v>
+      </c>
+      <c r="E1656" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1656" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G1656" t="n">
+        <v>243760</v>
+      </c>
+      <c r="H1656" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1656" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:52:49</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1657" t="n">
+        <v>252.01</v>
+      </c>
+      <c r="D1657" t="n">
+        <v>255</v>
+      </c>
+      <c r="E1657" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1657" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G1657" t="n">
+        <v>252010</v>
+      </c>
+      <c r="H1657" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1657" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>2026-08-06 11:47:26</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>SENSEX2680678500PE</t>
+        </is>
+      </c>
+      <c r="C1658" t="n">
+        <v>227.18</v>
+      </c>
+      <c r="D1658" t="n">
+        <v>230.2</v>
+      </c>
+      <c r="E1658" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F1658" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G1658" t="n">
+        <v>227180</v>
+      </c>
+      <c r="H1658" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1658" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>2026-08-07 12:16:03</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1659" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="D1659" t="n">
+        <v>121.7</v>
+      </c>
+      <c r="E1659" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1659" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G1659" t="n">
+        <v>140049</v>
+      </c>
+      <c r="H1659" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1659" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>2026-08-07 12:26:16</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1660" t="n">
+        <v>121.94</v>
+      </c>
+      <c r="D1660" t="n">
+        <v>113.58</v>
+      </c>
+      <c r="E1660" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1660" t="n">
+        <v>-9781.200000000001</v>
+      </c>
+      <c r="G1660" t="n">
+        <v>142669.8</v>
+      </c>
+      <c r="H1660" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1660" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>2026-08-07 12:46:42</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>NIFTY2681124500CE</t>
+        </is>
+      </c>
+      <c r="C1661" t="n">
+        <v>169.24</v>
+      </c>
+      <c r="D1661" t="n">
+        <v>174.25</v>
+      </c>
+      <c r="E1661" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1661" t="n">
+        <v>5861.7</v>
+      </c>
+      <c r="G1661" t="n">
+        <v>198010.8</v>
+      </c>
+      <c r="H1661" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1661" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>2026-08-07 13:01:39</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>NIFTY2681124600PE</t>
+        </is>
+      </c>
+      <c r="C1662" t="n">
+        <v>133.96</v>
+      </c>
+      <c r="D1662" t="n">
+        <v>136.45</v>
+      </c>
+      <c r="E1662" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1662" t="n">
+        <v>2913.3</v>
+      </c>
+      <c r="G1662" t="n">
+        <v>156733.2</v>
+      </c>
+      <c r="H1662" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1662" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>2026-08-07 13:25:46</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1663" t="n">
+        <v>112.88</v>
+      </c>
+      <c r="D1663" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="E1663" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1663" t="n">
+        <v>-10272.6</v>
+      </c>
+      <c r="G1663" t="n">
+        <v>132069.6</v>
+      </c>
+      <c r="H1663" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1663" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>2026-08-07 13:32:06</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1664" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="D1664" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="E1664" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1664" t="n">
+        <v>2925</v>
+      </c>
+      <c r="G1664" t="n">
+        <v>125307</v>
+      </c>
+      <c r="H1664" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1664" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>2026-08-07 13:34:29</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1665" t="n">
+        <v>111.86</v>
+      </c>
+      <c r="D1665" t="n">
+        <v>114.35</v>
+      </c>
+      <c r="E1665" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1665" t="n">
+        <v>2913.3</v>
+      </c>
+      <c r="G1665" t="n">
+        <v>130876.2</v>
+      </c>
+      <c r="H1665" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1665" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>2026-08-07 14:06:55</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550PE</t>
+        </is>
+      </c>
+      <c r="C1666" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="D1666" t="n">
+        <v>115</v>
+      </c>
+      <c r="E1666" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1666" t="n">
+        <v>2925</v>
+      </c>
+      <c r="G1666" t="n">
+        <v>131625</v>
+      </c>
+      <c r="H1666" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1666" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>2026-08-07 14:46:48</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550CE</t>
+        </is>
+      </c>
+      <c r="C1667" t="n">
+        <v>128.57</v>
+      </c>
+      <c r="D1667" t="n">
+        <v>131.05</v>
+      </c>
+      <c r="E1667" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1667" t="n">
+        <v>2901.6</v>
+      </c>
+      <c r="G1667" t="n">
+        <v>150426.9</v>
+      </c>
+      <c r="H1667" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1667" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:13:43</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>NIFTY2681124500CE</t>
+        </is>
+      </c>
+      <c r="C1668" t="n">
+        <v>163.09</v>
+      </c>
+      <c r="D1668" t="n">
+        <v>165.1</v>
+      </c>
+      <c r="E1668" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1668" t="n">
+        <v>2351.7</v>
+      </c>
+      <c r="G1668" t="n">
+        <v>190815.3</v>
+      </c>
+      <c r="H1668" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1668" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:15:35</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>NIFTY2681124500CE</t>
+        </is>
+      </c>
+      <c r="C1669" t="n">
+        <v>165.65</v>
+      </c>
+      <c r="D1669" t="n">
+        <v>167.65</v>
+      </c>
+      <c r="E1669" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1669" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G1669" t="n">
+        <v>193810.5</v>
+      </c>
+      <c r="H1669" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1669" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:20:18</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>NIFTY2681124500CE</t>
+        </is>
+      </c>
+      <c r="C1670" t="n">
+        <v>167.88</v>
+      </c>
+      <c r="D1670" t="n">
+        <v>169.9</v>
+      </c>
+      <c r="E1670" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1670" t="n">
+        <v>2363.4</v>
+      </c>
+      <c r="G1670" t="n">
+        <v>196419.6</v>
+      </c>
+      <c r="H1670" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1670" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:26:17</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>NIFTY2681124500CE</t>
+        </is>
+      </c>
+      <c r="C1671" t="n">
+        <v>169.78</v>
+      </c>
+      <c r="D1671" t="n">
+        <v>171.3</v>
+      </c>
+      <c r="E1671" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1671" t="n">
+        <v>1778.4</v>
+      </c>
+      <c r="G1671" t="n">
+        <v>198642.6</v>
+      </c>
+      <c r="H1671" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1671" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:13:09</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>NIFTY2681124700PE</t>
+        </is>
+      </c>
+      <c r="C1672" t="n">
+        <v>140.83</v>
+      </c>
+      <c r="D1672" t="n">
+        <v>127.61</v>
+      </c>
+      <c r="E1672" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1672" t="n">
+        <v>-15467.4</v>
+      </c>
+      <c r="G1672" t="n">
+        <v>164771.1</v>
+      </c>
+      <c r="H1672" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1672" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:16:43</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>NIFTY2681124600CE</t>
+        </is>
+      </c>
+      <c r="C1673" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="D1673" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="E1673" t="n">
+        <v>1755</v>
+      </c>
+      <c r="F1673" t="n">
+        <v>8775</v>
+      </c>
+      <c r="G1673" t="n">
+        <v>174096</v>
+      </c>
+      <c r="H1673" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1673" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:18:15</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>NIFTY2681124600CE</t>
+        </is>
+      </c>
+      <c r="C1674" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="D1674" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="E1674" t="n">
+        <v>1755</v>
+      </c>
+      <c r="F1674" t="n">
+        <v>5265</v>
+      </c>
+      <c r="G1674" t="n">
+        <v>181642.5</v>
+      </c>
+      <c r="H1674" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1674" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>2026-08-10 13:30:59</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550CE</t>
+        </is>
+      </c>
+      <c r="C1675" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="D1675" t="n">
+        <v>119.2</v>
+      </c>
+      <c r="E1675" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1675" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G1675" t="n">
+        <v>167596</v>
+      </c>
+      <c r="H1675" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1675" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>2026-08-10 13:33:14</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550CE</t>
+        </is>
+      </c>
+      <c r="C1676" t="n">
+        <v>119.95</v>
+      </c>
+      <c r="D1676" t="n">
+        <v>121.95</v>
+      </c>
+      <c r="E1676" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1676" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G1676" t="n">
+        <v>171528.5</v>
+      </c>
+      <c r="H1676" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1676" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>2026-08-10 13:34:18</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>NIFTY2681124550CE</t>
+        </is>
+      </c>
+      <c r="C1677" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="D1677" t="n">
+        <v>124.1</v>
+      </c>
+      <c r="E1677" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1677" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G1677" t="n">
+        <v>174603</v>
+      </c>
+      <c r="H1677" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1677" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>2026-08-11 12:57:49</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>NIFTY2681124600PE</t>
+        </is>
+      </c>
+      <c r="C1678" t="n">
+        <v>151.24</v>
+      </c>
+      <c r="D1678" t="n">
+        <v>153.25</v>
+      </c>
+      <c r="E1678" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1678" t="n">
+        <v>2874.3</v>
+      </c>
+      <c r="G1678" t="n">
+        <v>216273.2</v>
+      </c>
+      <c r="H1678" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1678" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:05:50</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>NIFTY2681124350CE</t>
+        </is>
+      </c>
+      <c r="C1679" t="n">
+        <v>128.45</v>
+      </c>
+      <c r="D1679" t="n">
+        <v>130.45</v>
+      </c>
+      <c r="E1679" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1679" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G1679" t="n">
+        <v>183683.5</v>
+      </c>
+      <c r="H1679" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1679" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:08:22</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>NIFTY2681124350CE</t>
+        </is>
+      </c>
+      <c r="C1680" t="n">
+        <v>128.92</v>
+      </c>
+      <c r="D1680" t="n">
+        <v>130.9</v>
+      </c>
+      <c r="E1680" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1680" t="n">
+        <v>2831.4</v>
+      </c>
+      <c r="G1680" t="n">
+        <v>184355.6</v>
+      </c>
+      <c r="H1680" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1680" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:11:32</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>NIFTY2681124350CE</t>
+        </is>
+      </c>
+      <c r="C1681" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="D1681" t="n">
+        <v>124.65</v>
+      </c>
+      <c r="E1681" t="n">
+        <v>130</v>
+      </c>
+      <c r="F1681" t="n">
+        <v>-903.5</v>
+      </c>
+      <c r="G1681" t="n">
+        <v>17108</v>
+      </c>
+      <c r="H1681" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I1681" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:57:15</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>NIFTY2681124600PE</t>
+        </is>
+      </c>
+      <c r="C1682" t="n">
+        <v>138.28</v>
+      </c>
+      <c r="D1682" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="E1682" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F1682" t="n">
+        <v>2888.6</v>
+      </c>
+      <c r="G1682" t="n">
+        <v>197740.4</v>
+      </c>
+      <c r="H1682" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1682" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:52:23</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>SENSEX2682077400CE</t>
+        </is>
+      </c>
+      <c r="C1683" t="n">
+        <v>129.15</v>
+      </c>
+      <c r="D1683" t="n">
+        <v>132.65</v>
+      </c>
+      <c r="E1683" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F1683" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G1683" t="n">
+        <v>193725</v>
+      </c>
+      <c r="H1683" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1683" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:09:40</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>SENSEX2682077500PE</t>
+        </is>
+      </c>
+      <c r="C1684" t="n">
+        <v>114.4</v>
+      </c>
+      <c r="D1684" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="E1684" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F1684" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G1684" t="n">
+        <v>171600</v>
+      </c>
+      <c r="H1684" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I1684" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:37:57</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>NIFTY2691523250CE</t>
+        </is>
+      </c>
+      <c r="C1685" t="n">
+        <v>173.55</v>
+      </c>
+      <c r="D1685" t="n">
+        <v>175.2</v>
+      </c>
+      <c r="E1685" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1685" t="n">
+        <v>1930.5</v>
+      </c>
+      <c r="G1685" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:39:49</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>NIFTY2691523300CE</t>
+        </is>
+      </c>
+      <c r="C1686" t="n">
+        <v>138.1</v>
+      </c>
+      <c r="D1686" t="n">
+        <v>139.1</v>
+      </c>
+      <c r="E1686" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1686" t="n">
+        <v>1170</v>
+      </c>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:42:31</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1687" t="n">
+        <v>113.95</v>
+      </c>
+      <c r="D1687" t="n">
+        <v>114.95</v>
+      </c>
+      <c r="E1687" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1687" t="n">
+        <v>1170</v>
+      </c>
+      <c r="G1687" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:48:28</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350PE</t>
+        </is>
+      </c>
+      <c r="C1688" t="n">
+        <v>99.95</v>
+      </c>
+      <c r="D1688" t="n">
+        <v>101</v>
+      </c>
+      <c r="E1688" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1688" t="n">
+        <v>1228.5</v>
+      </c>
+      <c r="G1688" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:51:56</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>NIFTY2691523450PE</t>
+        </is>
+      </c>
+      <c r="C1689" t="n">
+        <v>158.55</v>
+      </c>
+      <c r="D1689" t="n">
+        <v>160.4</v>
+      </c>
+      <c r="E1689" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1689" t="n">
+        <v>2164.5</v>
+      </c>
+      <c r="G1689" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:53:34</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>NIFTY2691523300CE</t>
+        </is>
+      </c>
+      <c r="C1690" t="n">
+        <v>136.75</v>
+      </c>
+      <c r="D1690" t="n">
+        <v>138.4</v>
+      </c>
+      <c r="E1690" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1690" t="n">
+        <v>1930.5</v>
+      </c>
+      <c r="G1690" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:58:12</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1691" t="n">
+        <v>110</v>
+      </c>
+      <c r="D1691" t="n">
+        <v>111.6</v>
+      </c>
+      <c r="E1691" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1691" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G1691" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:59:04</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>NIFTY2691523450PE</t>
+        </is>
+      </c>
+      <c r="C1692" t="n">
+        <v>147.35</v>
+      </c>
+      <c r="D1692" t="n">
+        <v>148.95</v>
+      </c>
+      <c r="E1692" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1692" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G1692" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:00:03</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>NIFTY2691523500PE</t>
+        </is>
+      </c>
+      <c r="C1693" t="n">
+        <v>182.3</v>
+      </c>
+      <c r="D1693" t="n">
+        <v>183.9</v>
+      </c>
+      <c r="E1693" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1693" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G1693" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:02:13</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>NIFTY2691523450PE</t>
+        </is>
+      </c>
+      <c r="C1694" t="n">
+        <v>155.25</v>
+      </c>
+      <c r="D1694" t="n">
+        <v>157</v>
+      </c>
+      <c r="E1694" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1694" t="n">
+        <v>2047.5</v>
+      </c>
+      <c r="G1694" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:03:14</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350PE</t>
+        </is>
+      </c>
+      <c r="C1695" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="D1695" t="n">
+        <v>101.25</v>
+      </c>
+      <c r="E1695" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1695" t="n">
+        <v>1813.5</v>
+      </c>
+      <c r="G1695" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:04:37</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350PE</t>
+        </is>
+      </c>
+      <c r="C1696" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="D1696" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="E1696" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1696" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G1696" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:05:32</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350PE</t>
+        </is>
+      </c>
+      <c r="C1697" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D1697" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="E1697" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1697" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G1697" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:07:06</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1698" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="D1698" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="E1698" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1698" t="n">
+        <v>2223</v>
+      </c>
+      <c r="G1698" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:09:15</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>NIFTY2691523500PE</t>
+        </is>
+      </c>
+      <c r="C1699" t="n">
+        <v>198.15</v>
+      </c>
+      <c r="D1699" t="n">
+        <v>200.4</v>
+      </c>
+      <c r="E1699" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1699" t="n">
+        <v>2632.5</v>
+      </c>
+      <c r="G1699" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:10:20</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>NIFTY2691523300CE</t>
+        </is>
+      </c>
+      <c r="C1700" t="n">
+        <v>125.4</v>
+      </c>
+      <c r="D1700" t="n">
+        <v>127</v>
+      </c>
+      <c r="E1700" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1700" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G1700" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:13:06</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>NIFTY2691523300CE</t>
+        </is>
+      </c>
+      <c r="C1701" t="n">
+        <v>127.75</v>
+      </c>
+      <c r="D1701" t="n">
+        <v>129.25</v>
+      </c>
+      <c r="E1701" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1701" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G1701" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:15:31</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350PE</t>
+        </is>
+      </c>
+      <c r="C1702" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="D1702" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="E1702" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1702" t="n">
+        <v>2164.5</v>
+      </c>
+      <c r="G1702" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:18:57</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>NIFTY2691523400PE</t>
+        </is>
+      </c>
+      <c r="C1703" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="D1703" t="n">
+        <v>133.15</v>
+      </c>
+      <c r="E1703" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1703" t="n">
+        <v>1813.5</v>
+      </c>
+      <c r="G1703" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:20:48</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>NIFTY2691523400PE</t>
+        </is>
+      </c>
+      <c r="C1704" t="n">
+        <v>134.2</v>
+      </c>
+      <c r="D1704" t="n">
+        <v>135.85</v>
+      </c>
+      <c r="E1704" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1704" t="n">
+        <v>1930.5</v>
+      </c>
+      <c r="G1704" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:22:30</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>NIFTY2691523250CE</t>
+        </is>
+      </c>
+      <c r="C1705" t="n">
+        <v>157.95</v>
+      </c>
+      <c r="D1705" t="n">
+        <v>159.7</v>
+      </c>
+      <c r="E1705" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1705" t="n">
+        <v>2047.5</v>
+      </c>
+      <c r="G1705" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:32:36</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>NIFTY2691523450PE</t>
+        </is>
+      </c>
+      <c r="C1706" t="n">
+        <v>160.15</v>
+      </c>
+      <c r="D1706" t="n">
+        <v>145.5</v>
+      </c>
+      <c r="E1706" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1706" t="n">
+        <v>-17140.5</v>
+      </c>
+      <c r="G1706" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:33:35</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>NIFTY2691523400PE</t>
+        </is>
+      </c>
+      <c r="C1707" t="n">
+        <v>119.45</v>
+      </c>
+      <c r="D1707" t="n">
+        <v>121.25</v>
+      </c>
+      <c r="E1707" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1707" t="n">
+        <v>2106</v>
+      </c>
+      <c r="G1707" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:34:30</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>NIFTY2691523500PE</t>
+        </is>
+      </c>
+      <c r="C1708" t="n">
+        <v>186.75</v>
+      </c>
+      <c r="D1708" t="n">
+        <v>188.4</v>
+      </c>
+      <c r="E1708" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1708" t="n">
+        <v>1930.5</v>
+      </c>
+      <c r="G1708" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:39:57</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>NIFTY2691523400PE</t>
+        </is>
+      </c>
+      <c r="C1709" t="n">
+        <v>126.65</v>
+      </c>
+      <c r="D1709" t="n">
+        <v>128.65</v>
+      </c>
+      <c r="E1709" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1709" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G1709" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:42:18</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>NIFTY2691523200CE</t>
+        </is>
+      </c>
+      <c r="C1710" t="n">
+        <v>184.15</v>
+      </c>
+      <c r="D1710" t="n">
+        <v>186</v>
+      </c>
+      <c r="E1710" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1710" t="n">
+        <v>2164.5</v>
+      </c>
+      <c r="G1710" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:43:16</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1711" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="D1711" t="n">
+        <v>100.75</v>
+      </c>
+      <c r="E1711" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1711" t="n">
+        <v>2106</v>
+      </c>
+      <c r="G1711" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:50:33</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1712" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="D1712" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="E1712" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1712" t="n">
+        <v>1813.5</v>
+      </c>
+      <c r="G1712" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:51:39</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1713" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="D1713" t="n">
+        <v>106</v>
+      </c>
+      <c r="E1713" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1713" t="n">
+        <v>2398.5</v>
+      </c>
+      <c r="G1713" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:54:21</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>NIFTY2691523450PE</t>
+        </is>
+      </c>
+      <c r="C1714" t="n">
+        <v>153.3</v>
+      </c>
+      <c r="D1714" t="n">
+        <v>136.9</v>
+      </c>
+      <c r="E1714" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1714" t="n">
+        <v>-19188</v>
+      </c>
+      <c r="G1714" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:55:51</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>NIFTY2691523500PE</t>
+        </is>
+      </c>
+      <c r="C1715" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D1715" t="n">
+        <v>161</v>
+      </c>
+      <c r="E1715" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1715" t="n">
+        <v>-22756.5</v>
+      </c>
+      <c r="G1715" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:56:39</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>NIFTY2691523350CE</t>
+        </is>
+      </c>
+      <c r="C1716" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="D1716" t="n">
+        <v>125.6</v>
+      </c>
+      <c r="E1716" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1716" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G1716" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:58:44</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>NIFTY2691523400PE</t>
+        </is>
+      </c>
+      <c r="C1717" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="D1717" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="E1717" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F1717" t="n">
+        <v>3042</v>
+      </c>
+      <c r="G1717" t="inlineStr">
+        <is>
+          <t>MOMENTUM_BOT</t>
         </is>
       </c>
     </row>

</xml_diff>